<commit_message>
Update CI workflow and Selenium test files
</commit_message>
<xml_diff>
--- a/auralis-selenium-real/Auralis_Test_Report.xlsx
+++ b/auralis-selenium-real/Auralis_Test_Report.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Test Results" sheetId="1" r:id="rId1"/>
+    <sheet name="E2E Test Report" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,23 +397,38 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:G19"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="29.83203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="4" max="4" width="44.83203125" customWidth="1"/>
+    <col min="5" max="5" width="21.83203125" customWidth="1"/>
+    <col min="6" max="6" width="9.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Test ID</v>
       </c>
       <c r="B1" t="str">
-        <v>Test Name</v>
+        <v>Test File</v>
       </c>
       <c r="C1" t="str">
-        <v>Expected Result</v>
+        <v>Test Suite</v>
       </c>
       <c r="D1" t="str">
-        <v>Actual Result</v>
+        <v>Test Case</v>
       </c>
       <c r="E1" t="str">
+        <v>Duration (Seconds)</v>
+      </c>
+      <c r="F1" t="str">
         <v>Status</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Actual Result / Error</v>
       </c>
     </row>
     <row r="2">
@@ -421,16 +436,22 @@
         <v>TC001</v>
       </c>
       <c r="B2" t="str">
-        <v>Smoke Test</v>
+        <v>dashboard.test.js</v>
       </c>
       <c r="C2" t="str">
-        <v>Application should open</v>
+        <v>Dashboard Test</v>
       </c>
       <c r="D2" t="str">
-        <v>Application opened successfully</v>
+        <v>should login and reach dashboard</v>
       </c>
       <c r="E2" t="str">
-        <v>PASS</v>
+        <v>13.48</v>
+      </c>
+      <c r="F2" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Verified successfully</v>
       </c>
     </row>
     <row r="3">
@@ -438,16 +459,22 @@
         <v>TC002</v>
       </c>
       <c r="B3" t="str">
-        <v>Login Test</v>
+        <v>dashboard.test.js</v>
       </c>
       <c r="C3" t="str">
-        <v>User should login successfully</v>
+        <v>Dashboard Test</v>
       </c>
       <c r="D3" t="str">
-        <v>Login successful</v>
+        <v>should display dashboard content</v>
       </c>
       <c r="E3" t="str">
-        <v>PASS</v>
+        <v>5.46</v>
+      </c>
+      <c r="F3" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Verified successfully</v>
       </c>
     </row>
     <row r="4">
@@ -455,16 +482,22 @@
         <v>TC003</v>
       </c>
       <c r="B4" t="str">
-        <v>Dashboard Test</v>
+        <v>emergency-services.test.js</v>
       </c>
       <c r="C4" t="str">
-        <v>Dashboard should load</v>
+        <v>Emergency Services Test</v>
       </c>
       <c r="D4" t="str">
-        <v>Dashboard loaded successfully</v>
+        <v>should verify emergency numbers</v>
       </c>
       <c r="E4" t="str">
-        <v>PASS</v>
+        <v>13.25</v>
+      </c>
+      <c r="F4" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Verified successfully</v>
       </c>
     </row>
     <row r="5">
@@ -472,16 +505,22 @@
         <v>TC004</v>
       </c>
       <c r="B5" t="str">
-        <v>Navigation Test</v>
+        <v>guardian.test.js</v>
       </c>
       <c r="C5" t="str">
-        <v>Navigation routes should work</v>
+        <v>Guardian Network Test</v>
       </c>
       <c r="D5" t="str">
-        <v>Map, Chat, Notifications, Profile accessible</v>
+        <v>should open Guardian Network page</v>
       </c>
       <c r="E5" t="str">
-        <v>PASS</v>
+        <v>15.08</v>
+      </c>
+      <c r="F5" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Verified successfully</v>
       </c>
     </row>
     <row r="6">
@@ -489,16 +528,22 @@
         <v>TC005</v>
       </c>
       <c r="B6" t="str">
-        <v>Notifications Test</v>
+        <v>login.test.js</v>
       </c>
       <c r="C6" t="str">
-        <v>Notifications page should display alerts</v>
+        <v>Auralis Login Test</v>
       </c>
       <c r="D6" t="str">
-        <v>Safety Alert, AI Safety Tip, Check-in Reminder displayed</v>
+        <v>should login successfully</v>
       </c>
       <c r="E6" t="str">
-        <v>PASS</v>
+        <v>14.62</v>
+      </c>
+      <c r="F6" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Verified successfully</v>
       </c>
     </row>
     <row r="7">
@@ -506,16 +551,22 @@
         <v>TC006</v>
       </c>
       <c r="B7" t="str">
-        <v>Profile Test</v>
+        <v>module-discovery.test.js</v>
       </c>
       <c r="C7" t="str">
-        <v>Profile page should load</v>
+        <v>Module Discovery</v>
       </c>
       <c r="D7" t="str">
-        <v>Profile details and emergency contacts displayed</v>
+        <v>should discover all buttons</v>
       </c>
       <c r="E7" t="str">
-        <v>PASS</v>
+        <v>11.45</v>
+      </c>
+      <c r="F7" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Verified successfully</v>
       </c>
     </row>
     <row r="8">
@@ -523,16 +574,22 @@
         <v>TC007</v>
       </c>
       <c r="B8" t="str">
-        <v>Emergency Services Test</v>
+        <v>modules.test.js</v>
       </c>
       <c r="C8" t="str">
-        <v>Emergency numbers should be visible</v>
+        <v>Dashboard Modules Test</v>
       </c>
       <c r="D8" t="str">
-        <v>100, 108, 101, 1091 verified</v>
+        <v>should verify all dashboard modules exist</v>
       </c>
       <c r="E8" t="str">
-        <v>PASS</v>
+        <v>11.06</v>
+      </c>
+      <c r="F8" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Verified successfully</v>
       </c>
     </row>
     <row r="9">
@@ -540,16 +597,22 @@
         <v>TC008</v>
       </c>
       <c r="B9" t="str">
-        <v>SOS Feature Test</v>
+        <v>navigation.test.js</v>
       </c>
       <c r="C9" t="str">
-        <v>SOS button should be present</v>
+        <v>Navigation Test</v>
       </c>
       <c r="D9" t="str">
-        <v>SOS Hold-to-Activate button found</v>
+        <v>should login</v>
       </c>
       <c r="E9" t="str">
-        <v>PASS</v>
+        <v>11.38</v>
+      </c>
+      <c r="F9" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Verified successfully</v>
       </c>
     </row>
     <row r="10">
@@ -557,16 +620,22 @@
         <v>TC009</v>
       </c>
       <c r="B10" t="str">
-        <v>Route Discovery Test</v>
+        <v>navigation.test.js</v>
       </c>
       <c r="C10" t="str">
-        <v>Application routes should be identified</v>
+        <v>Navigation Test</v>
       </c>
       <c r="D10" t="str">
-        <v>Home, Map, Chat, Alerts, Profile discovered</v>
+        <v>should navigate to Map page</v>
       </c>
       <c r="E10" t="str">
-        <v>PASS</v>
+        <v>5.40</v>
+      </c>
+      <c r="F10" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Verified successfully</v>
       </c>
     </row>
     <row r="11">
@@ -574,16 +643,22 @@
         <v>TC010</v>
       </c>
       <c r="B11" t="str">
-        <v>Module Discovery Test</v>
+        <v>navigation.test.js</v>
       </c>
       <c r="C11" t="str">
-        <v>Dashboard modules should exist</v>
+        <v>Navigation Test</v>
       </c>
       <c r="D11" t="str">
-        <v>Journey, Guardian, Analytics, Incidents, Modes, Community, Report found</v>
+        <v>should navigate to Chat page</v>
       </c>
       <c r="E11" t="str">
-        <v>PASS</v>
+        <v>5.60</v>
+      </c>
+      <c r="F11" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Verified successfully</v>
       </c>
     </row>
     <row r="12">
@@ -591,16 +666,22 @@
         <v>TC011</v>
       </c>
       <c r="B12" t="str">
-        <v>Dashboard Modules Validation</v>
+        <v>navigation.test.js</v>
       </c>
       <c r="C12" t="str">
-        <v>All dashboard modules should be available</v>
+        <v>Navigation Test</v>
       </c>
       <c r="D12" t="str">
-        <v>All modules verified successfully</v>
+        <v>should navigate to Notifications page</v>
       </c>
       <c r="E12" t="str">
-        <v>PASS</v>
+        <v>5.69</v>
+      </c>
+      <c r="F12" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Verified successfully</v>
       </c>
     </row>
     <row r="13">
@@ -608,21 +689,165 @@
         <v>TC012</v>
       </c>
       <c r="B13" t="str">
-        <v>Settings Validation</v>
+        <v>navigation.test.js</v>
       </c>
       <c r="C13" t="str">
-        <v>Settings page should exist</v>
+        <v>Navigation Test</v>
       </c>
       <c r="D13" t="str">
-        <v>No separate settings page; integrated into Profile</v>
+        <v>should navigate to Profile page</v>
       </c>
       <c r="E13" t="str">
-        <v>INFO</v>
+        <v>5.38</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Verified successfully</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>notifications.test.js</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Notifications Test</v>
+      </c>
+      <c r="D14" t="str">
+        <v>should open notifications page</v>
+      </c>
+      <c r="E14" t="str">
+        <v>15.61</v>
+      </c>
+      <c r="F14" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Verified successfully</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>profile.test.js</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Profile Test</v>
+      </c>
+      <c r="D15" t="str">
+        <v>should open profile page</v>
+      </c>
+      <c r="E15" t="str">
+        <v>16.43</v>
+      </c>
+      <c r="F15" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Verified successfully</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>route-discovery.test.js</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Route Discovery</v>
+      </c>
+      <c r="D16" t="str">
+        <v>should discover links</v>
+      </c>
+      <c r="E16" t="str">
+        <v>11.37</v>
+      </c>
+      <c r="F16" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Verified successfully</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>settings.test.js</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Settings Test</v>
+      </c>
+      <c r="D17" t="str">
+        <v>should check for settings section</v>
+      </c>
+      <c r="E17" t="str">
+        <v>17.07</v>
+      </c>
+      <c r="F17" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Verified successfully</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>smoke.test.js</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Auralis Smoke Test</v>
+      </c>
+      <c r="D18" t="str">
+        <v>should open Auralis website</v>
+      </c>
+      <c r="E18" t="str">
+        <v>6.01</v>
+      </c>
+      <c r="F18" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Verified successfully</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>sos.test.js</v>
+      </c>
+      <c r="C19" t="str">
+        <v>SOS Test</v>
+      </c>
+      <c r="D19" t="str">
+        <v>should login and inspect all SOS buttons</v>
+      </c>
+      <c r="E19" t="str">
+        <v>21.07</v>
+      </c>
+      <c r="F19" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Verified successfully</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>